<commit_message>
Enhance environment configuration and infrastructure setup for Phase 2. Updated `.env.example` with PostgreSQL and MinIO settings, including new database names and ports. Modified `docker-compose.yml` for PostgreSQL and MinIO services, ensuring compatibility with the new configurations. Updated `.gitignore` to manage Airflow logs and added documentation in `README.md` and `PROGRESS.md` to reflect current phase requirements and infrastructure details.
</commit_message>
<xml_diff>
--- a/docs/PROJECT_WBS.xlsx
+++ b/docs/PROJECT_WBS.xlsx
@@ -4987,7 +4987,7 @@
       </c>
       <c r="J75" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K75" s="56">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="J76" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K76" s="56">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="J77" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K77" s="56">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="J78" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K78" s="56">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="J79" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K79" s="56">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="J80" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K80" s="56">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="J81" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K81" s="56">
@@ -5400,7 +5400,7 @@
       </c>
       <c r="J82" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K82" s="56">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="J83" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K83" s="56">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="J84" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K84" s="56">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="J85" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K85" s="56">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="J86" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K86" s="56">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="J87" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K87" s="56">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="J88" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K88" s="56">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="J89" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K89" s="56">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="J90" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K90" s="56">
@@ -28729,7 +28729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N93"/>
+  <dimension ref="A1:N93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -28748,6 +28748,7 @@
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
@@ -28762,6 +28763,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="42" t="inlineStr">
         <is>
@@ -28846,6 +28848,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="51" t="inlineStr">
         <is>
@@ -29497,7 +29501,7 @@
       </c>
       <c r="J19" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K19" s="56">
@@ -29556,7 +29560,7 @@
       </c>
       <c r="J20" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K20" s="56">
@@ -29615,7 +29619,7 @@
       </c>
       <c r="J21" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="K21" s="56">
@@ -29674,7 +29678,7 @@
       </c>
       <c r="J22" s="38" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DOING</t>
         </is>
       </c>
       <c r="K22" s="56">

</xml_diff>